<commit_message>
fixed it_0_ recheck results
</commit_message>
<xml_diff>
--- a/Dataset Preprocessing Step 1.xlsx
+++ b/Dataset Preprocessing Step 1.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shariarimrozekhan/Documents/GitHub/masterThesis2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7631A703-B1E4-F94C-B8A2-B74AE05DDE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC7F6D99-D0BE-9B47-99F3-D1A2EA884B39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-6800" yWindow="-28200" windowWidth="51200" windowHeight="26240" xr2:uid="{34B6D257-D5DC-C445-8CB9-ED13F757CC8C}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="20060" xr2:uid="{34B6D257-D5DC-C445-8CB9-ED13F757CC8C}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset Preprocessing " sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -177,9 +176,6 @@
     <t>CASENO</t>
   </si>
   <si>
-    <t>900k Reports</t>
-  </si>
-  <si>
     <t>30k Reports</t>
   </si>
   <si>
@@ -192,19 +188,22 @@
     <t>Comments</t>
   </si>
   <si>
-    <t xml:space="preserve">Renamed in 900k Reports. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Renamed in 30k Reports. </t>
-  </si>
-  <si>
     <t xml:space="preserve">Delete from 30k. </t>
   </si>
   <si>
-    <t xml:space="preserve">Column Missing. Added column in 30K Reports. </t>
-  </si>
-  <si>
     <t>28k Reports</t>
+  </si>
+  <si>
+    <t>700k Reports</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rename in 700k Reports. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rename in 30k Reports. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Column Missing. Add column in 30K Reports. </t>
   </si>
 </sst>
 </file>
@@ -311,59 +310,13 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -394,13 +347,14 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="16"/>
+        <sz val="12"/>
         <color theme="1"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -440,6 +394,44 @@
       </font>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -454,17 +446,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{01D7D729-B805-EE49-86A2-C3B8EF7B3736}" name="Table1" displayName="Table1" ref="A1:F44" totalsRowShown="0" headerRowDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{01D7D729-B805-EE49-86A2-C3B8EF7B3736}" name="Table1" displayName="Table1" ref="A1:F44" totalsRowShown="0" headerRowDxfId="6">
   <autoFilter ref="A1:F44" xr:uid="{01D7D729-B805-EE49-86A2-C3B8EF7B3736}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{430CACE4-363E-AB4B-B88B-494C71BAB737}" name="14k Reports" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{28603752-3ECD-924C-876A-19777147A8FA}" name="28k Reports" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{430CACE4-363E-AB4B-B88B-494C71BAB737}" name="14k Reports" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{28603752-3ECD-924C-876A-19777147A8FA}" name="28k Reports" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{B6FDD917-83B8-024A-AA8C-EFECAB980D5F}" name="30k Reports"/>
-    <tableColumn id="3" xr3:uid="{2F502FA8-08E0-2642-A368-00516DFF6A6A}" name="900k Reports" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{2AC988D3-90AE-A040-8DFD-69C585AD2B1A}" name="Match?" dataDxfId="1">
+    <tableColumn id="3" xr3:uid="{2F502FA8-08E0-2642-A368-00516DFF6A6A}" name="700k Reports" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{2AC988D3-90AE-A040-8DFD-69C585AD2B1A}" name="Match?" dataDxfId="2">
       <calculatedColumnFormula>AND(EXACT(A2,B2), EXACT(B2,C2), EXACT(C2,D2))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7F4CAF21-F952-3F4D-B718-A813FB2C7D07}" name="Comments" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{7F4CAF21-F952-3F4D-B718-A813FB2C7D07}" name="Comments" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -791,32 +783,32 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.1640625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="50" style="3" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="45.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="39.83203125" style="3" customWidth="1"/>
     <col min="4" max="4" width="36.1640625" style="3" customWidth="1"/>
     <col min="5" max="5" width="46.5" style="3" customWidth="1"/>
-    <col min="6" max="6" width="30.33203125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="41" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="16384" width="10.83203125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.2">
       <c r="A1" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="C1" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="D1" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="E1" s="14" t="s">
+      <c r="F1" s="14" t="s">
         <v>49</v>
-      </c>
-      <c r="F1" s="14" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1093,7 +1085,9 @@
       <c r="A17" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="2"/>
+      <c r="B17" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="C17" s="13" t="s">
         <v>18</v>
       </c>
@@ -1105,7 +1099,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1144,7 +1138,7 @@
         <v>0</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1237,7 +1231,7 @@
         <v>0</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="34" x14ac:dyDescent="0.2">
@@ -1256,7 +1250,7 @@
         <v>0</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1282,7 +1276,7 @@
         <v>16</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C27" s="13" t="s">
         <v>16</v>
@@ -1292,7 +1286,7 @@
       </c>
       <c r="E27" s="2" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1300,7 +1294,7 @@
         <v>15</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C28" s="13" t="s">
         <v>15</v>
@@ -1310,15 +1304,15 @@
       </c>
       <c r="E28" s="2" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
         <v>14</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>14</v>
@@ -1328,7 +1322,7 @@
       </c>
       <c r="E29" s="2" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1336,7 +1330,7 @@
         <v>12</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C30" s="13" t="s">
         <v>12</v>
@@ -1346,15 +1340,15 @@
       </c>
       <c r="E30" s="2" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>11</v>
@@ -1364,7 +1358,7 @@
       </c>
       <c r="E31" s="2" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1372,7 +1366,7 @@
         <v>10</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C32" s="13" t="s">
         <v>10</v>
@@ -1382,7 +1376,7 @@
       </c>
       <c r="E32" s="2" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1390,7 +1384,7 @@
         <v>9</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C33" s="13" t="s">
         <v>9</v>
@@ -1400,7 +1394,7 @@
       </c>
       <c r="E33" s="2" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1408,7 +1402,7 @@
         <v>8</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>8</v>
@@ -1418,7 +1412,7 @@
       </c>
       <c r="E34" s="2" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1426,7 +1420,7 @@
         <v>7</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>7</v>
@@ -1436,15 +1430,15 @@
       </c>
       <c r="E35" s="2" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>6</v>
@@ -1454,15 +1448,15 @@
       </c>
       <c r="E36" s="2" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>6</v>
+      <c r="B37" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>5</v>
@@ -1472,14 +1466,12 @@
       </c>
       <c r="E37" s="2" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
-      <c r="B38" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="B38" s="2"/>
       <c r="C38" s="5" t="s">
         <v>13</v>
       </c>
@@ -1489,7 +1481,7 @@
         <v>0</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
@@ -1504,7 +1496,7 @@
         <v>0</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -1519,7 +1511,7 @@
         <v>0</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
@@ -1534,7 +1526,7 @@
         <v>0</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
@@ -1549,7 +1541,7 @@
         <v>0</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
@@ -1564,7 +1556,7 @@
         <v>0</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
@@ -1579,7 +1571,7 @@
         <v>0</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1594,13 +1586,4 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FCA42A1-1609-2C48-8285-2411273555F0}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>